<commit_message>
changed mfn format: removed explanatory lines 2 and 3 from excel files added reading of speed via new fleets sheet
</commit_message>
<xml_diff>
--- a/tests/formats/mfn_excel/MFN_changed_order.xlsx
+++ b/tests/formats/mfn_excel/MFN_changed_order.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="DieseArbeitsmappe"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hess\Documents\C1_Work\C19_MediCar\medicar-vehicle-routing\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\en986\Documents\Projects\Alltours\generalized_agv_path_finding\tests\formats\mfn_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AB90607-D82A-4EA0-913A-A88FA5411F31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80B0E1C7-7689-4F28-A3EE-196AAEED6FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="831" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30612" yWindow="228" windowWidth="30936" windowHeight="16776" tabRatio="831" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="19" r:id="rId1"/>
@@ -26,7 +26,7 @@
     <sheet name="ElevatorsComplex" sheetId="47" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">NetworkNodes!$A$1:$P$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">NetworkNodes!$A$1:$K$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
@@ -606,7 +606,7 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -626,17 +626,15 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="18">
     <cellStyle name="Gut 2" xfId="16" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Komma 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Komma 3" xfId="15" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Prozent 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
     <cellStyle name="Prozent 3" xfId="8" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
     <cellStyle name="Prozent 3 2" xfId="12" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
     <cellStyle name="Standard 2 2" xfId="6" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
     <cellStyle name="Standard 2 2 2" xfId="11" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
@@ -927,7 +925,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Tabelle1"/>
   <dimension ref="A1:C31"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" customWidth="1"/>
     <col min="2" max="2" width="14.44140625" customWidth="1"/>
@@ -1106,7 +1104,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C9B3FFE-5E30-4A5C-AC25-2588E6856685}">
   <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
@@ -1137,7 +1135,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58E964F2-FF69-4819-A7C3-85CD51F2295C}">
   <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
@@ -1188,7 +1186,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C52C50EA-D3CE-4A3D-A603-A0E0539C6C86}">
   <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="13.44140625" bestFit="1" customWidth="1"/>
@@ -1246,7 +1244,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{159E6FE9-79AA-439F-A731-7339FCC4326E}">
   <dimension ref="A1:N4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="8.44140625" bestFit="1" customWidth="1"/>
@@ -1267,151 +1265,151 @@
         <v>7</v>
       </c>
       <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G1" t="s">
+        <v>84</v>
+      </c>
+      <c r="H1" t="s">
+        <v>85</v>
+      </c>
+      <c r="I1" t="s">
+        <v>86</v>
+      </c>
+      <c r="J1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L1" t="s">
         <v>22</v>
       </c>
-      <c r="C1" t="s">
+      <c r="M1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N1" t="s">
         <v>23</v>
-      </c>
-      <c r="D1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F1" t="s">
-        <v>87</v>
-      </c>
-      <c r="G1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H1" t="s">
-        <v>32</v>
-      </c>
-      <c r="I1" t="s">
-        <v>83</v>
-      </c>
-      <c r="J1" t="s">
-        <v>84</v>
-      </c>
-      <c r="K1" t="s">
-        <v>85</v>
-      </c>
-      <c r="L1" t="s">
-        <v>86</v>
-      </c>
-      <c r="M1" t="s">
-        <v>10</v>
-      </c>
-      <c r="N1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="16">
+      <c r="B2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2">
+        <v>5</v>
+      </c>
+      <c r="I2">
+        <v>5</v>
+      </c>
+      <c r="J2" t="s">
+        <v>117</v>
+      </c>
+      <c r="L2" s="16">
         <v>20</v>
       </c>
-      <c r="C2" s="16">
+      <c r="M2" s="16">
+        <v>0</v>
+      </c>
+      <c r="N2" s="16">
         <v>30</v>
-      </c>
-      <c r="D2" s="16">
-        <v>0</v>
-      </c>
-      <c r="E2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" t="s">
-        <v>82</v>
-      </c>
-      <c r="G2" t="s">
-        <v>88</v>
-      </c>
-      <c r="I2" t="s">
-        <v>33</v>
-      </c>
-      <c r="J2" t="s">
-        <v>33</v>
-      </c>
-      <c r="K2">
-        <v>5</v>
-      </c>
-      <c r="L2">
-        <v>5</v>
-      </c>
-      <c r="M2" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="16">
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" t="s">
+        <v>31</v>
+      </c>
+      <c r="J3" t="s">
+        <v>119</v>
+      </c>
+      <c r="L3" s="16">
         <v>50</v>
       </c>
-      <c r="C3" s="16">
+      <c r="M3" s="16">
+        <v>0</v>
+      </c>
+      <c r="N3" s="16">
         <v>30</v>
-      </c>
-      <c r="D3" s="16">
-        <v>0</v>
-      </c>
-      <c r="E3" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" t="s">
-        <v>26</v>
-      </c>
-      <c r="G3" t="s">
-        <v>88</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-      <c r="I3" t="s">
-        <v>31</v>
-      </c>
-      <c r="J3" t="s">
-        <v>31</v>
-      </c>
-      <c r="M3" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="16">
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" t="s">
+        <v>31</v>
+      </c>
+      <c r="J4" t="s">
+        <v>120</v>
+      </c>
+      <c r="L4" s="16">
         <v>80</v>
       </c>
-      <c r="C4" s="16">
+      <c r="M4" s="16">
+        <v>0</v>
+      </c>
+      <c r="N4" s="16">
         <v>30</v>
-      </c>
-      <c r="D4" s="16">
-        <v>0</v>
-      </c>
-      <c r="E4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G4" t="s">
-        <v>88</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4" t="s">
-        <v>31</v>
-      </c>
-      <c r="J4" t="s">
-        <v>31</v>
-      </c>
-      <c r="M4" t="s">
-        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -1422,7 +1420,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17E172D1-D225-4CD4-9721-555476AB5029}">
   <dimension ref="A1:N5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.88671875" bestFit="1" customWidth="1"/>
@@ -1593,7 +1591,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C00FCB5D-D806-47EA-B7BD-35B4F00A2E0F}">
   <dimension ref="A1:N1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.5546875" bestFit="1" customWidth="1"/>
@@ -1661,8 +1659,8 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81F5D0D1-03B0-4AAD-AB55-5A9935202F87}">
-  <dimension ref="A1:X3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:X2"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.109375" customWidth="1"/>
     <col min="2" max="4" width="22.5546875" customWidth="1"/>
@@ -1686,25 +1684,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+      <c r="A1" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" t="s">
         <v>110</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" t="s">
         <v>111</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" t="s">
         <v>49</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" t="s">
         <v>127</v>
       </c>
-      <c r="G1" s="17" t="s">
+      <c r="G1" t="s">
         <v>50</v>
       </c>
       <c r="H1" t="s">
@@ -1760,25 +1758,25 @@
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A2" s="17" t="s">
+      <c r="A2" t="s">
         <v>112</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" t="s">
         <v>113</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" t="s">
         <v>125</v>
       </c>
-      <c r="D2" s="17">
+      <c r="D2">
         <v>2</v>
       </c>
-      <c r="E2" s="17">
+      <c r="E2">
         <v>1</v>
       </c>
-      <c r="F2" s="17">
+      <c r="F2">
         <v>0.5</v>
       </c>
-      <c r="G2" s="17">
+      <c r="G2">
         <v>0.5</v>
       </c>
       <c r="H2">
@@ -1826,15 +1824,6 @@
       <c r="W2" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A3" s="18"/>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -1845,7 +1834,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBE8010C-4AB8-4C54-9235-5FBF88DCB2DF}">
   <dimension ref="A1:K5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5" bestFit="1" customWidth="1"/>
@@ -2012,7 +2001,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E324AC1-F817-40ED-8A3A-986A3543B34E}">
   <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="26.109375" customWidth="1"/>
     <col min="3" max="4" width="20.109375" customWidth="1"/>
@@ -2048,7 +2037,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFF82848-22FB-4F29-A247-2C4A188888ED}">
   <dimension ref="A1:P1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.109375" bestFit="1" customWidth="1"/>
   </cols>
@@ -2249,18 +2238,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2282,14 +2271,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22FFC1BB-A9F9-4CC6-ADBD-2FE4E08E51F6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D3FF907-6B7B-4F23-94BF-42A9560A2884}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -2303,4 +2284,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22FFC1BB-A9F9-4CC6-ADBD-2FE4E08E51F6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>